<commit_message>
Paper-data from field-trail added
Added written data during field aplication of cattle-slury 28-10-2025
</commit_message>
<xml_diff>
--- a/Lab acidification field & lab comparision/Soil-sample IDs.xlsx
+++ b/Lab acidification field & lab comparision/Soil-sample IDs.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab acidification field &amp; lab comparision\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E921A5-6F61-410F-B780-8EAA8564330B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ark1" sheetId="1" r:id="rId1"/>
+    <sheet name="Cattle-slurry" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,8 +24,22 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>Samples were scrapped on the bottom</t>
+  </si>
+  <si>
+    <t>Uneven surfaces on the top was kept</t>
+  </si>
+  <si>
+    <t>spots without too much plant-material was selected</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -49,8 +69,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +351,196 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="44.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1">
+        <v>47051</v>
+      </c>
+      <c r="C1">
+        <v>7201</v>
+      </c>
+      <c r="D1">
+        <v>7325</v>
+      </c>
+      <c r="E1">
+        <v>7219</v>
+      </c>
+      <c r="F1">
+        <v>7385</v>
+      </c>
+      <c r="G1">
+        <v>7407</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>7334</v>
+      </c>
+      <c r="D2">
+        <v>7326</v>
+      </c>
+      <c r="E2">
+        <v>7211</v>
+      </c>
+      <c r="F2">
+        <v>7393</v>
+      </c>
+      <c r="G2">
+        <v>7403</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>7209</v>
+      </c>
+      <c r="D3">
+        <v>7346</v>
+      </c>
+      <c r="E3">
+        <v>7381</v>
+      </c>
+      <c r="F3">
+        <v>7390</v>
+      </c>
+      <c r="G3">
+        <v>7406</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>7342</v>
+      </c>
+      <c r="D4">
+        <v>7331</v>
+      </c>
+      <c r="E4">
+        <v>7382</v>
+      </c>
+      <c r="F4">
+        <v>7391</v>
+      </c>
+      <c r="G4">
+        <v>7405</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <v>7204</v>
+      </c>
+      <c r="D5">
+        <v>7328</v>
+      </c>
+      <c r="E5">
+        <v>7383</v>
+      </c>
+      <c r="F5">
+        <v>7387</v>
+      </c>
+      <c r="G5">
+        <v>7394</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>7338</v>
+      </c>
+      <c r="D6">
+        <v>7349</v>
+      </c>
+      <c r="E6">
+        <v>7384</v>
+      </c>
+      <c r="F6">
+        <v>7394</v>
+      </c>
+      <c r="G6">
+        <v>7400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C7">
+        <v>7335</v>
+      </c>
+      <c r="D7">
+        <v>7350</v>
+      </c>
+      <c r="E7">
+        <v>7388</v>
+      </c>
+      <c r="F7">
+        <v>7395</v>
+      </c>
+      <c r="G7">
+        <v>7397</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C8">
+        <v>7327</v>
+      </c>
+      <c r="D8">
+        <v>7345</v>
+      </c>
+      <c r="E8">
+        <v>7392</v>
+      </c>
+      <c r="F8">
+        <v>7402</v>
+      </c>
+      <c r="G8">
+        <v>7404</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <v>7348</v>
+      </c>
+      <c r="D9">
+        <v>7221</v>
+      </c>
+      <c r="E9">
+        <v>7389</v>
+      </c>
+      <c r="F9">
+        <v>7401</v>
+      </c>
+      <c r="G9">
+        <v>7396</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C10">
+        <v>7330</v>
+      </c>
+      <c r="D10">
+        <v>7347</v>
+      </c>
+      <c r="E10">
+        <v>7386</v>
+      </c>
+      <c r="F10">
+        <v>7408</v>
+      </c>
+      <c r="G10">
+        <v>7398</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>